<commit_message>
- Organized the folders, especially the one from baseline models - Updated LFCC + Delta baseline model - Added the other models (with different features) using the LFCC as a base
</commit_message>
<xml_diff>
--- a/Training_Results_Template_with_Charts.xlsx
+++ b/Training_Results_Template_with_Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Felipe\Team Lab\teamlab-phonetics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66D880E-5F2E-423F-8C02-CF1E964F76DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1645FD60-137B-49DB-9B29-AB6A34B3949D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Training Results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>Feature Type</t>
   </si>
@@ -101,13 +101,16 @@
   </si>
   <si>
     <t>256 h. dimensions / Precision: 0.7413 / Recall: 0.9614</t>
+  </si>
+  <si>
+    <t>Threshold Validation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +122,18 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -156,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -173,11 +188,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -869,7 +890,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>609599</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -900,7 +921,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -933,7 +954,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -968,10 +989,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrainingResults" displayName="TrainingResults" ref="A1:L10" headerRowDxfId="2">
-  <autoFilter ref="A1:L10" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="12">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Feature Type" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrainingResults" displayName="TrainingResults" ref="A1:M10" headerRowDxfId="3">
+  <autoFilter ref="A1:M10" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="13">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Feature Type" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Model Architecture"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="# Samples"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Patience"/>
@@ -982,7 +1003,8 @@
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="F1 Score"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Accuracy (%)"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Additional Info"/>
-    <tableColumn id="1" xr3:uid="{241E01D4-BC5E-46D0-964C-94B99384C214}" name="EER Training/Validation" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{241E01D4-BC5E-46D0-964C-94B99384C214}" name="EER Training/Validation" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{30CDF536-98B5-4854-BC84-021C336CB0F9}" name="Threshold Validation" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1273,23 +1295,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" customWidth="1"/>
-    <col min="9" max="9" width="13.77734375" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="50.88671875" customWidth="1"/>
-    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="11" max="11" width="50.85546875" customWidth="1"/>
+    <col min="12" max="13" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1326,8 +1348,11 @@
       <c r="L1" s="4" t="s">
         <v>20</v>
       </c>
+      <c r="M1" s="6" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1342,8 +1367,9 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1358,8 +1384,9 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1374,8 +1401,9 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1408,8 +1436,9 @@
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -1424,8 +1453,9 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1440,8 +1470,9 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1478,8 +1509,9 @@
       <c r="L8" s="1">
         <v>0.31</v>
       </c>
+      <c r="M8" s="1"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1516,8 +1548,9 @@
       <c r="L9" s="1">
         <v>1.99</v>
       </c>
+      <c r="M9" s="1"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
@@ -1554,8 +1587,10 @@
       <c r="L10" s="1">
         <v>1.28</v>
       </c>
+      <c r="M10" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>